<commit_message>
📅 日报更新 2026-09-02 03:04
</commit_message>
<xml_diff>
--- a/data/exports/黄老师/dist_order_2026-09-02.xlsx
+++ b/data/exports/黄老师/dist_order_2026-09-02.xlsx
@@ -125,11 +125,11 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="0">
-        <v>49887876</v>
+        <v>49937566</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>鱼靖儿</t>
+          <t>简单sincerity</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -154,7 +154,7 @@
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:23:11</t>
+          <t>2026-09-02 10:10:33</t>
         </is>
       </c>
       <c r="H2" s="0" t="inlineStr">
@@ -164,7 +164,7 @@
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J2" s="0" t="inlineStr">
@@ -185,11 +185,11 @@
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="0">
-        <v>49887478</v>
+        <v>49937187</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>风调雨顺</t>
+          <t>莲子</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -214,7 +214,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:10:17</t>
+          <t>2026-09-02 09:58:56</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -224,7 +224,7 @@
       </c>
       <c r="I3" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J3" s="0" t="inlineStr">
@@ -245,11 +245,11 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="0">
-        <v>49887447</v>
+        <v>49937101</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>中国艺人</t>
+          <t>蓉儿</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -274,7 +274,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:44</t>
+          <t>2026-09-02 09:56:16</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -305,11 +305,11 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="0">
-        <v>49887439</v>
+        <v>49937098</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>黄晓玲</t>
+          <t>瀚林2368</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -334,7 +334,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:17</t>
+          <t>2026-09-02 09:56:15</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
@@ -365,11 +365,11 @@
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="0">
-        <v>49887437</v>
+        <v>49937081</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>随缘</t>
+          <t>🔱 花中之美</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -394,7 +394,7 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:07</t>
+          <t>2026-09-02 09:55:47</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
@@ -425,11 +425,11 @@
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="0">
-        <v>49887416</v>
+        <v>49937066</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>刘秋红</t>
+          <t>雨情</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -454,7 +454,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:31</t>
+          <t>2026-09-02 09:55:27</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
@@ -485,11 +485,11 @@
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="0">
-        <v>49887403</v>
+        <v>49937061</v>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>Mr.</t>
+          <t>Sunny 🎈瑶</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -514,7 +514,7 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:05</t>
+          <t>2026-09-02 09:55:23</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
@@ -545,11 +545,11 @@
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="0">
-        <v>49887401</v>
+        <v>49887876</v>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>万事如意</t>
+          <t>鱼靖儿</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:03</t>
+          <t>2026-08-31 23:23:11</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
@@ -605,11 +605,11 @@
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="0">
-        <v>49887400</v>
+        <v>49887478</v>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>💋诺墨</t>
+          <t>风调雨顺</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:01</t>
+          <t>2026-08-31 23:10:17</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
@@ -665,11 +665,11 @@
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="0">
-        <v>49887399</v>
+        <v>49887447</v>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>听风</t>
+          <t>中国艺人</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:06:59</t>
+          <t>2026-08-31 23:08:44</t>
         </is>
       </c>
       <c r="H11" s="0" t="inlineStr">
@@ -725,11 +725,11 @@
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="0">
-        <v>49845584</v>
+        <v>49887439</v>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>彭汉平13024282926</t>
+          <t>黄晓玲</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:18:55</t>
+          <t>2026-08-31 23:08:17</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
@@ -785,11 +785,11 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="0">
-        <v>49845487</v>
+        <v>49887437</v>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>Z国华</t>
+          <t>随缘</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:15:49</t>
+          <t>2026-08-31 23:08:07</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="I13" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J13" s="0" t="inlineStr">
@@ -845,11 +845,11 @@
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="0">
-        <v>49845407</v>
+        <v>49887416</v>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>月亮🌛</t>
+          <t>刘秋红</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:12:33</t>
+          <t>2026-08-31 23:07:31</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
@@ -905,11 +905,11 @@
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="0">
-        <v>49845398</v>
+        <v>49887403</v>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>老树</t>
+          <t>Mr.</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:12:03</t>
+          <t>2026-08-31 23:07:05</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
@@ -965,11 +965,11 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="0">
-        <v>49845391</v>
+        <v>49887401</v>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>八哥</t>
+          <t>万事如意</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:45</t>
+          <t>2026-08-31 23:07:03</t>
         </is>
       </c>
       <c r="H16" s="0" t="inlineStr">
@@ -1025,11 +1025,11 @@
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="0">
-        <v>49845380</v>
+        <v>49887400</v>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>铲车主出租15352562068</t>
+          <t>💋诺墨</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:29</t>
+          <t>2026-08-31 23:07:01</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
@@ -1085,11 +1085,11 @@
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="0">
-        <v>49845376</v>
+        <v>49887399</v>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>刘萍</t>
+          <t>听风</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:15</t>
+          <t>2026-08-31 23:06:59</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
@@ -1145,11 +1145,11 @@
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="0">
-        <v>49845374</v>
+        <v>49845584</v>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>空谷幽兰</t>
+          <t>彭汉平13024282926</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:07</t>
+          <t>2026-08-30 23:18:55</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
@@ -1205,11 +1205,11 @@
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="0">
-        <v>49845373</v>
+        <v>49845487</v>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>泽浩羊</t>
+          <t>Z国华</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:05</t>
+          <t>2026-08-30 23:15:49</t>
         </is>
       </c>
       <c r="H20" s="0" t="inlineStr">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J20" s="0" t="inlineStr">
@@ -1265,11 +1265,11 @@
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="0">
-        <v>49845367</v>
+        <v>49845407</v>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>峰回路转</t>
+          <t>月亮🌛</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:55</t>
+          <t>2026-08-30 23:12:33</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
@@ -1325,11 +1325,11 @@
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="0">
-        <v>49845366</v>
+        <v>49845398</v>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>超儿</t>
+          <t>老树</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:51</t>
+          <t>2026-08-30 23:12:03</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
@@ -1385,11 +1385,11 @@
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="0">
-        <v>49845365</v>
+        <v>49845391</v>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>传</t>
+          <t>八哥</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:49</t>
+          <t>2026-08-30 23:11:45</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
@@ -1445,11 +1445,11 @@
     </row>
     <row r="24" spans="1:14">
       <c r="A24" s="0">
-        <v>49845360</v>
+        <v>49845380</v>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>悟歌</t>
+          <t>铲车主出租15352562068</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:43</t>
+          <t>2026-08-30 23:11:29</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
@@ -1505,11 +1505,11 @@
     </row>
     <row r="25" spans="1:14">
       <c r="A25" s="0">
-        <v>49845342</v>
+        <v>49845376</v>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>丽丽</t>
+          <t>刘萍</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:15</t>
+          <t>2026-08-30 23:11:15</t>
         </is>
       </c>
       <c r="H25" s="0" t="inlineStr">
@@ -1565,11 +1565,11 @@
     </row>
     <row r="26" spans="1:14">
       <c r="A26" s="0">
-        <v>49826011</v>
+        <v>49845374</v>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>王前卫</t>
+          <t>空谷幽兰</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:57:27</t>
+          <t>2026-08-30 23:11:07</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -1625,11 +1625,11 @@
     </row>
     <row r="27" spans="1:14">
       <c r="A27" s="0">
-        <v>49825720</v>
+        <v>49845373</v>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>老A</t>
+          <t>泽浩羊</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:46:02</t>
+          <t>2026-08-30 23:11:05</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
@@ -1685,11 +1685,11 @@
     </row>
     <row r="28" spans="1:14">
       <c r="A28" s="0">
-        <v>49825676</v>
+        <v>49845367</v>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>蓝天</t>
+          <t>峰回路转</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:44:05</t>
+          <t>2026-08-30 23:10:55</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
@@ -1745,11 +1745,11 @@
     </row>
     <row r="29" spans="1:14">
       <c r="A29" s="0">
-        <v>49825650</v>
+        <v>49845366</v>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>爱芳</t>
+          <t>超儿</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:43:11</t>
+          <t>2026-08-30 23:10:51</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
@@ -1805,11 +1805,11 @@
     </row>
     <row r="30" spans="1:14">
       <c r="A30" s="0">
-        <v>49825642</v>
+        <v>49845365</v>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>银杏树</t>
+          <t>传</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:55</t>
+          <t>2026-08-30 23:10:49</t>
         </is>
       </c>
       <c r="H30" s="0" t="inlineStr">
@@ -1865,11 +1865,11 @@
     </row>
     <row r="31" spans="1:14">
       <c r="A31" s="0">
-        <v>49825640</v>
+        <v>49845360</v>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>遵命有福（杨凤）</t>
+          <t>悟歌</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:49</t>
+          <t>2026-08-30 23:10:43</t>
         </is>
       </c>
       <c r="H31" s="0" t="inlineStr">
@@ -1925,11 +1925,11 @@
     </row>
     <row r="32" spans="1:14">
       <c r="A32" s="0">
-        <v>49825639</v>
+        <v>49845342</v>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>申华</t>
+          <t>丽丽</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:49</t>
+          <t>2026-08-30 23:10:15</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
@@ -1985,11 +1985,11 @@
     </row>
     <row r="33" spans="1:14">
       <c r="A33" s="0">
-        <v>49825637</v>
+        <v>49826011</v>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>陈月焓</t>
+          <t>王前卫</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:47</t>
+          <t>2026-08-30 12:57:27</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
@@ -2045,11 +2045,11 @@
     </row>
     <row r="34" spans="1:14">
       <c r="A34" s="0">
-        <v>49825635</v>
+        <v>49825720</v>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>小镇生活&amp;&amp;杜震</t>
+          <t>老A</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:43</t>
+          <t>2026-08-30 12:46:02</t>
         </is>
       </c>
       <c r="H34" s="0" t="inlineStr">
@@ -2105,11 +2105,11 @@
     </row>
     <row r="35" spans="1:14">
       <c r="A35" s="0">
-        <v>49825628</v>
+        <v>49825676</v>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>Taᴗaoᥫᩣ</t>
+          <t>蓝天</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:35</t>
+          <t>2026-08-30 12:44:05</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
@@ -2165,11 +2165,11 @@
     </row>
     <row r="36" spans="1:14">
       <c r="A36" s="0">
-        <v>49782066</v>
+        <v>49825650</v>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>前程似锦</t>
+          <t>爱芳</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 09:07:29</t>
+          <t>2026-08-30 12:43:11</t>
         </is>
       </c>
       <c r="H36" s="0" t="inlineStr">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="I36" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J36" s="0" t="inlineStr">
@@ -2225,11 +2225,11 @@
     </row>
     <row r="37" spans="1:14">
       <c r="A37" s="0">
-        <v>49771027</v>
+        <v>49825642</v>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>非比</t>
+          <t>银杏树</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 23:30:09</t>
+          <t>2026-08-30 12:42:55</t>
         </is>
       </c>
       <c r="H37" s="0" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="I37" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J37" s="0" t="inlineStr">
@@ -2285,11 +2285,11 @@
     </row>
     <row r="38" spans="1:14">
       <c r="A38" s="0">
-        <v>49673360</v>
+        <v>49825640</v>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>德行天下</t>
+          <t>遵命有福（杨凤）</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:19:03</t>
+          <t>2026-08-30 12:42:49</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="I38" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J38" s="0" t="inlineStr">
@@ -2345,11 +2345,11 @@
     </row>
     <row r="39" spans="1:14">
       <c r="A39" s="0">
-        <v>49673352</v>
+        <v>49825639</v>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>余盛将至2026</t>
+          <t>申华</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:49</t>
+          <t>2026-08-30 12:42:49</t>
         </is>
       </c>
       <c r="H39" s="0" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="I39" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J39" s="0" t="inlineStr">
@@ -2405,11 +2405,11 @@
     </row>
     <row r="40" spans="1:14">
       <c r="A40" s="0">
-        <v>49673350</v>
+        <v>49825637</v>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>山居客</t>
+          <t>陈月焓</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -2434,7 +2434,7 @@
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:47</t>
+          <t>2026-08-30 12:42:47</t>
         </is>
       </c>
       <c r="H40" s="0" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="I40" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J40" s="0" t="inlineStr">
@@ -2465,11 +2465,11 @@
     </row>
     <row r="41" spans="1:14">
       <c r="A41" s="0">
-        <v>49673349</v>
+        <v>49825635</v>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>白云</t>
+          <t>小镇生活&amp;&amp;杜震</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:45</t>
+          <t>2026-08-30 12:42:43</t>
         </is>
       </c>
       <c r="H41" s="0" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="I41" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J41" s="0" t="inlineStr">
@@ -2525,11 +2525,11 @@
     </row>
     <row r="42" spans="1:14">
       <c r="A42" s="0">
-        <v>49646935</v>
+        <v>49825628</v>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>马跃荣</t>
+          <t>Taᴗaoᥫᩣ</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:59</t>
+          <t>2026-08-30 12:42:35</t>
         </is>
       </c>
       <c r="H42" s="0" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="I42" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J42" s="0" t="inlineStr">
@@ -2585,11 +2585,11 @@
     </row>
     <row r="43" spans="1:14">
       <c r="A43" s="0">
-        <v>49646933</v>
+        <v>49782066</v>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>@吴</t>
+          <t>前程似锦</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:56</t>
+          <t>2026-08-29 09:07:29</t>
         </is>
       </c>
       <c r="H43" s="0" t="inlineStr">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="I43" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J43" s="0" t="inlineStr">
@@ -2645,11 +2645,11 @@
     </row>
     <row r="44" spans="1:14">
       <c r="A44" s="0">
-        <v>49646901</v>
+        <v>49771027</v>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>龙安：富华／</t>
+          <t>非比</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:14:28</t>
+          <t>2026-08-28 23:30:09</t>
         </is>
       </c>
       <c r="H44" s="0" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="I44" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J44" s="0" t="inlineStr">
@@ -2705,11 +2705,11 @@
     </row>
     <row r="45" spans="1:14">
       <c r="A45" s="0">
-        <v>49646876</v>
+        <v>49673360</v>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>冬日暖阳🌻</t>
+          <t>德行天下</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -2734,7 +2734,7 @@
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:37</t>
+          <t>2026-08-26 12:19:03</t>
         </is>
       </c>
       <c r="H45" s="0" t="inlineStr">
@@ -2765,11 +2765,11 @@
     </row>
     <row r="46" spans="1:14">
       <c r="A46" s="0">
-        <v>49646867</v>
+        <v>49673352</v>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>寒雨</t>
+          <t>余盛将至2026</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:15</t>
+          <t>2026-08-26 12:18:49</t>
         </is>
       </c>
       <c r="H46" s="0" t="inlineStr">
@@ -2825,11 +2825,11 @@
     </row>
     <row r="47" spans="1:14">
       <c r="A47" s="0">
-        <v>49636232</v>
+        <v>49673350</v>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>平安</t>
+          <t>山居客</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -2854,7 +2854,7 @@
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:20:15</t>
+          <t>2026-08-26 12:18:47</t>
         </is>
       </c>
       <c r="H47" s="0" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="I47" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J47" s="0" t="inlineStr">
@@ -2885,11 +2885,11 @@
     </row>
     <row r="48" spans="1:14">
       <c r="A48" s="0">
-        <v>49636184</v>
+        <v>49673349</v>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>古道西风</t>
+          <t>白云</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:55</t>
+          <t>2026-08-26 12:18:45</t>
         </is>
       </c>
       <c r="H48" s="0" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="I48" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J48" s="0" t="inlineStr">
@@ -2945,11 +2945,11 @@
     </row>
     <row r="49" spans="1:14">
       <c r="A49" s="0">
-        <v>49636170</v>
+        <v>49646935</v>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>周海龙</t>
+          <t>马跃荣</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -2974,7 +2974,7 @@
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:33</t>
+          <t>2026-08-25 18:15:59</t>
         </is>
       </c>
       <c r="H49" s="0" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="I49" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J49" s="0" t="inlineStr">
@@ -3005,11 +3005,11 @@
     </row>
     <row r="50" spans="1:14">
       <c r="A50" s="0">
-        <v>49636157</v>
+        <v>49646933</v>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>锦妍</t>
+          <t>@吴</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:07</t>
+          <t>2026-08-25 18:15:56</t>
         </is>
       </c>
       <c r="H50" s="0" t="inlineStr">
@@ -3044,7 +3044,7 @@
       </c>
       <c r="I50" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J50" s="0" t="inlineStr">
@@ -3065,11 +3065,11 @@
     </row>
     <row r="51" spans="1:14">
       <c r="A51" s="0">
-        <v>49593974</v>
+        <v>49646901</v>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>兰兰</t>
+          <t>龙安：富华／</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -3094,7 +3094,7 @@
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:59:53</t>
+          <t>2026-08-25 18:14:28</t>
         </is>
       </c>
       <c r="H51" s="0" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="I51" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J51" s="0" t="inlineStr">
@@ -3125,11 +3125,11 @@
     </row>
     <row r="52" spans="1:14">
       <c r="A52" s="0">
-        <v>49593671</v>
+        <v>49646876</v>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>准备1号</t>
+          <t>冬日暖阳🌻</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -3154,7 +3154,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:49:27</t>
+          <t>2026-08-25 18:13:37</t>
         </is>
       </c>
       <c r="H52" s="0" t="inlineStr">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="I52" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J52" s="0" t="inlineStr">
@@ -3185,11 +3185,11 @@
     </row>
     <row r="53" spans="1:14">
       <c r="A53" s="0">
-        <v>49535916</v>
+        <v>49646867</v>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>真诚</t>
+          <t>寒雨</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:46:23</t>
+          <t>2026-08-25 18:13:15</t>
         </is>
       </c>
       <c r="H53" s="0" t="inlineStr">
@@ -3224,7 +3224,7 @@
       </c>
       <c r="I53" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J53" s="0" t="inlineStr">
@@ -3245,11 +3245,11 @@
     </row>
     <row r="54" spans="1:14">
       <c r="A54" s="0">
-        <v>49535653</v>
+        <v>49636232</v>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>如意家电13368134456维修</t>
+          <t>平安</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -3274,7 +3274,7 @@
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:28:25</t>
+          <t>2026-08-25 13:20:15</t>
         </is>
       </c>
       <c r="H54" s="0" t="inlineStr">
@@ -3305,11 +3305,11 @@
     </row>
     <row r="55" spans="1:14">
       <c r="A55" s="0">
-        <v>49535650</v>
+        <v>49636184</v>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>莺莺</t>
+          <t>古道西风</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:27:55</t>
+          <t>2026-08-25 13:18:55</t>
         </is>
       </c>
       <c r="H55" s="0" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="I55" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J55" s="0" t="inlineStr">
@@ -3360,21 +3360,16 @@
       <c r="L55" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N55" s="0" t="inlineStr">
-        <is>
-          <t>黄浦</t>
         </is>
       </c>
     </row>
     <row r="56" spans="1:14">
       <c r="A56" s="0">
-        <v>49508265</v>
+        <v>49636170</v>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>爱猫🐱 咪</t>
+          <t>周海龙</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -3399,7 +3394,7 @@
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 09:53:41</t>
+          <t>2026-08-25 13:18:33</t>
         </is>
       </c>
       <c r="H56" s="0" t="inlineStr">
@@ -3409,7 +3404,7 @@
       </c>
       <c r="I56" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J56" s="0" t="inlineStr">
@@ -3430,11 +3425,11 @@
     </row>
     <row r="57" spans="1:14">
       <c r="A57" s="0">
-        <v>49493414</v>
+        <v>49636157</v>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>惠平</t>
+          <t>锦妍</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -3459,7 +3454,7 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:53:02</t>
+          <t>2026-08-25 13:18:07</t>
         </is>
       </c>
       <c r="H57" s="0" t="inlineStr">
@@ -3469,7 +3464,7 @@
       </c>
       <c r="I57" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J57" s="0" t="inlineStr">
@@ -3490,11 +3485,11 @@
     </row>
     <row r="58" spans="1:14">
       <c r="A58" s="0">
-        <v>49493126</v>
+        <v>49593974</v>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>刘盼昭</t>
+          <t>兰兰</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -3519,7 +3514,7 @@
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:44:53</t>
+          <t>2026-08-24 12:59:53</t>
         </is>
       </c>
       <c r="H58" s="0" t="inlineStr">
@@ -3550,11 +3545,11 @@
     </row>
     <row r="59" spans="1:14">
       <c r="A59" s="0">
-        <v>49492499</v>
+        <v>49593671</v>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>红霞</t>
+          <t>准备1号</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -3579,7 +3574,7 @@
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:29:43</t>
+          <t>2026-08-24 12:49:27</t>
         </is>
       </c>
       <c r="H59" s="0" t="inlineStr">
@@ -3610,11 +3605,11 @@
     </row>
     <row r="60" spans="1:14">
       <c r="A60" s="0">
-        <v>49455301</v>
+        <v>49535916</v>
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>周开平</t>
+          <t>真诚</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -3639,7 +3634,7 @@
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 22:46:59</t>
+          <t>2026-08-22 23:46:23</t>
         </is>
       </c>
       <c r="H60" s="0" t="inlineStr">
@@ -3670,11 +3665,11 @@
     </row>
     <row r="61" spans="1:14">
       <c r="A61" s="0">
-        <v>49432023</v>
+        <v>49535653</v>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>花生米</t>
+          <t>如意家电13368134456维修</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -3699,7 +3694,7 @@
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 11:55:45</t>
+          <t>2026-08-22 23:28:25</t>
         </is>
       </c>
       <c r="H61" s="0" t="inlineStr">
@@ -3730,11 +3725,11 @@
     </row>
     <row r="62" spans="1:14">
       <c r="A62" s="0">
-        <v>49415939</v>
+        <v>49535650</v>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>杨梅芳</t>
+          <t>莺莺</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -3759,7 +3754,7 @@
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:58</t>
+          <t>2026-08-22 23:27:55</t>
         </is>
       </c>
       <c r="H62" s="0" t="inlineStr">
@@ -3769,32 +3764,37 @@
       </c>
       <c r="I62" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J62" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K62" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L62" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N62" s="0" t="inlineStr">
+        <is>
+          <t>黄浦</t>
         </is>
       </c>
     </row>
     <row r="63" spans="1:14">
       <c r="A63" s="0">
-        <v>49415918</v>
+        <v>49508265</v>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>心语无言</t>
+          <t>爱猫🐱 咪</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:24</t>
+          <t>2026-08-22 09:53:41</t>
         </is>
       </c>
       <c r="H63" s="0" t="inlineStr">
@@ -3829,17 +3829,17 @@
       </c>
       <c r="I63" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J63" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K63" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L63" s="0" t="inlineStr">
@@ -3850,11 +3850,11 @@
     </row>
     <row r="64" spans="1:14">
       <c r="A64" s="0">
-        <v>49415913</v>
+        <v>49493414</v>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>安好</t>
+          <t>惠平</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:18</t>
+          <t>2026-08-21 22:53:02</t>
         </is>
       </c>
       <c r="H64" s="0" t="inlineStr">
@@ -3889,17 +3889,17 @@
       </c>
       <c r="I64" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J64" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K64" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L64" s="0" t="inlineStr">
@@ -3910,11 +3910,11 @@
     </row>
     <row r="65" spans="1:14">
       <c r="A65" s="0">
-        <v>49415890</v>
+        <v>49493126</v>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>雨夜聆风</t>
+          <t>刘盼昭</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:56</t>
+          <t>2026-08-21 22:44:53</t>
         </is>
       </c>
       <c r="H65" s="0" t="inlineStr">
@@ -3949,37 +3949,32 @@
       </c>
       <c r="I65" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J65" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K65" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L65" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N65" s="0" t="inlineStr">
-        <is>
-          <t>宜春</t>
         </is>
       </c>
     </row>
     <row r="66" spans="1:14">
       <c r="A66" s="0">
-        <v>49415874</v>
+        <v>49492499</v>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>飘</t>
+          <t>红霞</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -4004,7 +3999,7 @@
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:40</t>
+          <t>2026-08-21 22:29:43</t>
         </is>
       </c>
       <c r="H66" s="0" t="inlineStr">
@@ -4014,17 +4009,17 @@
       </c>
       <c r="I66" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J66" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K66" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L66" s="0" t="inlineStr">
@@ -4035,11 +4030,11 @@
     </row>
     <row r="67" spans="1:14">
       <c r="A67" s="0">
-        <v>49415871</v>
+        <v>49455301</v>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>庆</t>
+          <t>周开平</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -4064,7 +4059,7 @@
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:36</t>
+          <t>2026-08-20 22:46:59</t>
         </is>
       </c>
       <c r="H67" s="0" t="inlineStr">
@@ -4074,17 +4069,17 @@
       </c>
       <c r="I67" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J67" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K67" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L67" s="0" t="inlineStr">
@@ -4095,59 +4090,484 @@
     </row>
     <row r="68" spans="1:14">
       <c r="A68" s="0">
+        <v>49432023</v>
+      </c>
+      <c r="B68" s="0" t="inlineStr">
+        <is>
+          <t>花生米</t>
+        </is>
+      </c>
+      <c r="C68" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D68" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E68" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F68" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G68" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-20 11:55:45</t>
+        </is>
+      </c>
+      <c r="H68" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I68" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J68" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K68" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L68" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" spans="1:14">
+      <c r="A69" s="0">
+        <v>49415939</v>
+      </c>
+      <c r="B69" s="0" t="inlineStr">
+        <is>
+          <t>杨梅芳</t>
+        </is>
+      </c>
+      <c r="C69" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D69" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E69" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F69" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G69" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:58</t>
+        </is>
+      </c>
+      <c r="H69" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I69" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J69" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K69" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L69" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" spans="1:14">
+      <c r="A70" s="0">
+        <v>49415918</v>
+      </c>
+      <c r="B70" s="0" t="inlineStr">
+        <is>
+          <t>心语无言</t>
+        </is>
+      </c>
+      <c r="C70" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D70" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F70" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G70" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:24</t>
+        </is>
+      </c>
+      <c r="H70" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I70" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J70" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K70" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L70" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" spans="1:14">
+      <c r="A71" s="0">
+        <v>49415913</v>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
+          <t>安好</t>
+        </is>
+      </c>
+      <c r="C71" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D71" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E71" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F71" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G71" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:18</t>
+        </is>
+      </c>
+      <c r="H71" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I71" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J71" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K71" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L71" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" spans="1:14">
+      <c r="A72" s="0">
+        <v>49415890</v>
+      </c>
+      <c r="B72" s="0" t="inlineStr">
+        <is>
+          <t>雨夜聆风</t>
+        </is>
+      </c>
+      <c r="C72" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D72" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E72" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F72" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G72" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:56</t>
+        </is>
+      </c>
+      <c r="H72" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I72" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J72" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K72" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L72" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="N72" s="0" t="inlineStr">
+        <is>
+          <t>宜春</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" spans="1:14">
+      <c r="A73" s="0">
+        <v>49415874</v>
+      </c>
+      <c r="B73" s="0" t="inlineStr">
+        <is>
+          <t>飘</t>
+        </is>
+      </c>
+      <c r="C73" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D73" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E73" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F73" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G73" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:40</t>
+        </is>
+      </c>
+      <c r="H73" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I73" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J73" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K73" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L73" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" spans="1:14">
+      <c r="A74" s="0">
+        <v>49415871</v>
+      </c>
+      <c r="B74" s="0" t="inlineStr">
+        <is>
+          <t>庆</t>
+        </is>
+      </c>
+      <c r="C74" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D74" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E74" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F74" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G74" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:36</t>
+        </is>
+      </c>
+      <c r="H74" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I74" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J74" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K74" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L74" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" spans="1:14">
+      <c r="A75" s="0">
         <v>49415867</v>
       </c>
-      <c r="B68" s="0" t="inlineStr">
+      <c r="B75" s="0" t="inlineStr">
         <is>
           <t>HYQ</t>
         </is>
       </c>
-      <c r="C68" s="0" t="inlineStr">
-        <is>
-          <t>6天0基础钢琴入门课</t>
-        </is>
-      </c>
-      <c r="D68" s="0" t="inlineStr">
-        <is>
-          <t>训练营</t>
-        </is>
-      </c>
-      <c r="E68" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="F68" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="G68" s="0" t="inlineStr">
+      <c r="C75" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D75" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E75" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F75" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G75" s="0" t="inlineStr">
         <is>
           <t>2026-08-19 22:47:33</t>
         </is>
       </c>
-      <c r="H68" s="0" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I68" s="0" t="inlineStr">
-        <is>
-          <t>黄老师-抖音01</t>
-        </is>
-      </c>
-      <c r="J68" s="0" t="inlineStr">
+      <c r="H75" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I75" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J75" s="0" t="inlineStr">
         <is>
           <t>安迪钢琴-多个点击报名-0元</t>
         </is>
       </c>
-      <c r="K68" s="0" t="inlineStr">
+      <c r="K75" s="0" t="inlineStr">
         <is>
           <t>微信支付</t>
         </is>
       </c>
-      <c r="L68" s="0" t="inlineStr">
+      <c r="L75" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>

</xml_diff>